<commit_message>
reimplemented form 700 data changes that got reverted
</commit_message>
<xml_diff>
--- a/data/form_700/sonoma_2021.xlsx
+++ b/data/form_700/sonoma_2021.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/david/local_csci/csc131_project/data/form_700/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDFF8A36-F06E-EC4B-A50A-FABB6D001795}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F3840D8-13D8-3142-AD82-BE1DDCC303A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="29020" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="660" yWindow="3520" windowWidth="29020" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Schedule A1" sheetId="2" r:id="rId1"/>
@@ -1175,7 +1175,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1613" uniqueCount="395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1613" uniqueCount="394">
   <si>
     <t>Last Name</t>
   </si>
@@ -2443,9 +2443,6 @@
     <t>Portfolia Consumer Fund</t>
   </si>
   <si>
-    <t>KEYS#Keysight Technologies Inc.</t>
-  </si>
-  <si>
     <t>ARC Healthcare</t>
   </si>
   <si>
@@ -2560,13 +2557,13 @@
     <t>Walmart#WMT</t>
   </si>
   <si>
-    <t>Walt Disney</t>
-  </si>
-  <si>
     <t>HPQ#Hewlett-Packard#Hewlett Packard</t>
   </si>
   <si>
-    <t>landpaths</t>
+    <t>KEYS#Keysight Technologies</t>
+  </si>
+  <si>
+    <t>Landpaths</t>
   </si>
 </sst>
 </file>
@@ -2796,10 +2793,10 @@
     <xf numFmtId="14" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3133,72 +3130,72 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="I1" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="J1" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="K1" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="13" t="s">
+      <c r="L1" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="13" t="s">
+      <c r="M1" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="13" t="s">
+      <c r="N1" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="13" t="s">
+      <c r="O1" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="13" t="s">
+      <c r="P1" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="13"/>
+      <c r="Q1" s="14"/>
     </row>
     <row r="2" spans="1:17">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="13"/>
-      <c r="K2" s="13"/>
-      <c r="L2" s="13"/>
-      <c r="M2" s="13"/>
-      <c r="N2" s="13"/>
-      <c r="O2" s="13"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14"/>
+      <c r="M2" s="14"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="14"/>
       <c r="P2" s="1" t="s">
         <v>16</v>
       </c>
@@ -3237,7 +3234,7 @@
         <v>44620.73710648148</v>
       </c>
       <c r="L3" s="11" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="M3" s="4" t="s">
         <v>25</v>
@@ -3282,7 +3279,7 @@
         <v>44620.73710648148</v>
       </c>
       <c r="L4" s="12" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="M4" s="7" t="s">
         <v>25</v>
@@ -3327,7 +3324,7 @@
         <v>44620.73710648148</v>
       </c>
       <c r="L5" s="12" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="M5" s="7" t="s">
         <v>25</v>
@@ -3372,7 +3369,7 @@
         <v>44620.73710648148</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>27</v>
@@ -3417,7 +3414,7 @@
         <v>44620.73710648148</v>
       </c>
       <c r="L7" s="12" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="M7" s="7" t="s">
         <v>25</v>
@@ -3507,7 +3504,7 @@
         <v>44620.73710648148</v>
       </c>
       <c r="L9" s="12" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="M9" s="7" t="s">
         <v>25</v>
@@ -3552,7 +3549,7 @@
         <v>44620.73710648148</v>
       </c>
       <c r="L10" s="12" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="M10" s="7" t="s">
         <v>31</v>
@@ -3597,7 +3594,7 @@
         <v>44620.73710648148</v>
       </c>
       <c r="L11" s="12" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="M11" s="7" t="s">
         <v>30</v>
@@ -3642,7 +3639,7 @@
         <v>44635.468206018515</v>
       </c>
       <c r="L12" s="7" t="s">
-        <v>392</v>
+        <v>105</v>
       </c>
       <c r="M12" s="7" t="s">
         <v>37</v>
@@ -3829,8 +3826,8 @@
       <c r="K16" s="6">
         <v>44628.593032407407</v>
       </c>
-      <c r="L16" s="12" t="s">
-        <v>353</v>
+      <c r="L16" s="7" t="s">
+        <v>392</v>
       </c>
       <c r="M16" s="7" t="s">
         <v>52</v>
@@ -3877,7 +3874,7 @@
         <v>44628.593032407407</v>
       </c>
       <c r="L17" s="12" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="M17" s="7" t="s">
         <v>52</v>
@@ -3924,7 +3921,7 @@
         <v>44628.593032407407</v>
       </c>
       <c r="L18" s="7" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
       <c r="M18" s="7" t="s">
         <v>52</v>
@@ -3971,7 +3968,7 @@
         <v>44628.593032407407</v>
       </c>
       <c r="L19" s="12" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="M19" s="7" t="s">
         <v>52</v>
@@ -4018,7 +4015,7 @@
         <v>44628.593032407407</v>
       </c>
       <c r="L20" s="7" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="M20" s="7" t="s">
         <v>52</v>
@@ -4065,7 +4062,7 @@
         <v>44628.593032407407</v>
       </c>
       <c r="L21" s="7" t="s">
-        <v>393</v>
+        <v>391</v>
       </c>
       <c r="M21" s="7" t="s">
         <v>52</v>
@@ -4110,7 +4107,7 @@
         <v>44615.621944444443</v>
       </c>
       <c r="L22" s="12" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="M22" s="7" t="s">
         <v>57</v>
@@ -4155,7 +4152,7 @@
         <v>44615.621944444443</v>
       </c>
       <c r="L23" s="12" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="M23" s="7" t="s">
         <v>58</v>
@@ -4245,7 +4242,7 @@
         <v>44615.621944444443</v>
       </c>
       <c r="L25" s="12" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="M25" s="7" t="s">
         <v>61</v>
@@ -4290,7 +4287,7 @@
         <v>44615.621944444443</v>
       </c>
       <c r="L26" s="12" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="M26" s="7" t="s">
         <v>62</v>
@@ -4335,7 +4332,7 @@
         <v>44615.621944444443</v>
       </c>
       <c r="L27" s="12" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="M27" s="7" t="s">
         <v>62</v>
@@ -4476,7 +4473,7 @@
         <v>44587.558275462958</v>
       </c>
       <c r="L30" s="12" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="M30" s="7" t="s">
         <v>75</v>
@@ -4523,7 +4520,7 @@
         <v>44587.558275462958</v>
       </c>
       <c r="L31" s="12" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="M31" s="7" t="s">
         <v>76</v>
@@ -4568,7 +4565,7 @@
         <v>44572.604270833333</v>
       </c>
       <c r="L32" s="12" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="M32" s="7" t="s">
         <v>82</v>
@@ -4613,7 +4610,7 @@
         <v>44631.713113425925</v>
       </c>
       <c r="L33" s="12" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="M33" s="7" t="s">
         <v>88</v>
@@ -4658,7 +4655,7 @@
         <v>44631.713113425925</v>
       </c>
       <c r="L34" s="12" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="M34" s="7" t="s">
         <v>44</v>
@@ -4703,7 +4700,7 @@
         <v>44631.713113425925</v>
       </c>
       <c r="L35" s="12" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="M35" s="7" t="s">
         <v>89</v>
@@ -4928,7 +4925,7 @@
         <v>44631.713113425925</v>
       </c>
       <c r="L40" s="7" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
       <c r="M40" s="7" t="s">
         <v>44</v>
@@ -4973,7 +4970,7 @@
         <v>44631.713113425925</v>
       </c>
       <c r="L41" s="7" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="M41" s="7" t="s">
         <v>97</v>
@@ -5063,7 +5060,7 @@
         <v>44631.713113425925</v>
       </c>
       <c r="L43" s="12" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="M43" s="7" t="s">
         <v>44</v>
@@ -5108,7 +5105,7 @@
         <v>44631.713113425925</v>
       </c>
       <c r="L44" s="12" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="M44" s="7" t="s">
         <v>99</v>
@@ -5243,7 +5240,7 @@
         <v>44631.713113425925</v>
       </c>
       <c r="L47" s="7" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="M47" s="7" t="s">
         <v>103</v>
@@ -5288,7 +5285,7 @@
         <v>44631.713113425925</v>
       </c>
       <c r="L48" s="12" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="M48" s="7" t="s">
         <v>104</v>
@@ -5423,7 +5420,7 @@
         <v>44631.713113425925</v>
       </c>
       <c r="L51" s="12" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="M51" s="7" t="s">
         <v>109</v>
@@ -5491,28 +5488,28 @@
       <c r="B53" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="L53" s="14" t="s">
-        <v>394</v>
+      <c r="L53" s="13" t="s">
+        <v>393</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="16">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="J1:J2"/>
     <mergeCell ref="K1:K2"/>
     <mergeCell ref="P1:Q1"/>
     <mergeCell ref="L1:L2"/>
     <mergeCell ref="M1:M2"/>
     <mergeCell ref="N1:N2"/>
     <mergeCell ref="O1:O2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="J1:J2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.2" top="0.12013890000000001" bottom="0" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape"/>
@@ -5572,142 +5569,142 @@
       <c r="I1" s="9"/>
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
-      <c r="L1" s="13" t="s">
+      <c r="L1" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="M1" s="13"/>
-      <c r="N1" s="13"/>
-      <c r="O1" s="13"/>
-      <c r="P1" s="13"/>
-      <c r="Q1" s="13"/>
-      <c r="R1" s="13"/>
-      <c r="S1" s="13"/>
+      <c r="M1" s="14"/>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
+      <c r="R1" s="14"/>
+      <c r="S1" s="14"/>
       <c r="T1" s="1" t="s">
         <v>113</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="V1" s="13" t="s">
+      <c r="V1" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="W1" s="13"/>
-      <c r="X1" s="13"/>
-      <c r="Y1" s="13"/>
-      <c r="Z1" s="13"/>
-      <c r="AA1" s="13"/>
-      <c r="AB1" s="13"/>
-      <c r="AC1" s="13"/>
-      <c r="AD1" s="13"/>
+      <c r="W1" s="14"/>
+      <c r="X1" s="14"/>
+      <c r="Y1" s="14"/>
+      <c r="Z1" s="14"/>
+      <c r="AA1" s="14"/>
+      <c r="AB1" s="14"/>
+      <c r="AC1" s="14"/>
+      <c r="AD1" s="14"/>
     </row>
     <row r="2" spans="1:30">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="G2" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="13" t="s">
+      <c r="I2" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="13" t="s">
+      <c r="J2" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="13" t="s">
+      <c r="K2" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="13" t="s">
+      <c r="L2" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="M2" s="13" t="s">
+      <c r="M2" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="N2" s="13" t="s">
+      <c r="N2" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="O2" s="13" t="s">
+      <c r="O2" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="P2" s="13" t="s">
+      <c r="P2" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" s="13"/>
-      <c r="R2" s="13" t="s">
+      <c r="Q2" s="14"/>
+      <c r="R2" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="S2" s="13" t="s">
+      <c r="S2" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="T2" s="13" t="s">
+      <c r="T2" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="U2" s="13" t="s">
+      <c r="U2" s="14" t="s">
         <v>123</v>
       </c>
-      <c r="V2" s="13" t="s">
+      <c r="V2" s="14" t="s">
         <v>124</v>
       </c>
-      <c r="W2" s="13"/>
-      <c r="X2" s="13" t="s">
+      <c r="W2" s="14"/>
+      <c r="X2" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="Y2" s="13"/>
-      <c r="Z2" s="13" t="s">
+      <c r="Y2" s="14"/>
+      <c r="Z2" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="AA2" s="13" t="s">
+      <c r="AA2" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="AB2" s="13"/>
-      <c r="AC2" s="13" t="s">
+      <c r="AB2" s="14"/>
+      <c r="AC2" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="AD2" s="13"/>
+      <c r="AD2" s="14"/>
     </row>
     <row r="3" spans="1:30" ht="25">
-      <c r="A3" s="13"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
-      <c r="L3" s="13"/>
-      <c r="M3" s="13"/>
-      <c r="N3" s="13"/>
-      <c r="O3" s="13"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
+      <c r="L3" s="14"/>
+      <c r="M3" s="14"/>
+      <c r="N3" s="14"/>
+      <c r="O3" s="14"/>
       <c r="P3" s="1" t="s">
         <v>16</v>
       </c>
       <c r="Q3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="R3" s="13"/>
-      <c r="S3" s="13"/>
-      <c r="T3" s="13"/>
-      <c r="U3" s="13"/>
+      <c r="R3" s="14"/>
+      <c r="S3" s="14"/>
+      <c r="T3" s="14"/>
+      <c r="U3" s="14"/>
       <c r="V3" s="1" t="s">
         <v>127</v>
       </c>
@@ -5720,7 +5717,7 @@
       <c r="Y3" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="Z3" s="13"/>
+      <c r="Z3" s="14"/>
       <c r="AA3" s="1" t="s">
         <v>16</v>
       </c>
@@ -6435,7 +6432,7 @@
         <v>44783.347083912035</v>
       </c>
       <c r="L14" s="12" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="M14" s="7" t="s">
         <v>164</v>
@@ -6767,7 +6764,7 @@
         <v>44935.525719872683</v>
       </c>
       <c r="L19" s="12" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="M19" s="7" t="s">
         <v>180</v>
@@ -6833,7 +6830,7 @@
         <v>44572.604270833333</v>
       </c>
       <c r="L20" s="12" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="M20" s="7" t="s">
         <v>185</v>
@@ -6899,7 +6896,7 @@
         <v>44572.604270833333</v>
       </c>
       <c r="L21" s="12" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="M21" s="7" t="s">
         <v>185</v>
@@ -6936,6 +6933,23 @@
     </row>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:J3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="AA2:AB2"/>
+    <mergeCell ref="R2:R3"/>
+    <mergeCell ref="S2:S3"/>
+    <mergeCell ref="T2:T3"/>
+    <mergeCell ref="U2:U3"/>
+    <mergeCell ref="V2:W2"/>
     <mergeCell ref="L1:S1"/>
     <mergeCell ref="V1:AD1"/>
     <mergeCell ref="L2:L3"/>
@@ -6946,23 +6960,6 @@
     <mergeCell ref="X2:Y2"/>
     <mergeCell ref="Z2:Z3"/>
     <mergeCell ref="AC2:AD2"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="AA2:AB2"/>
-    <mergeCell ref="R2:R3"/>
-    <mergeCell ref="S2:S3"/>
-    <mergeCell ref="T2:T3"/>
-    <mergeCell ref="U2:U3"/>
-    <mergeCell ref="V2:W2"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:J3"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.2" top="0.12013890000000001" bottom="0" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape"/>
@@ -7041,99 +7038,99 @@
       <c r="AA1" s="9"/>
     </row>
     <row r="2" spans="1:27">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="G2" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="13" t="s">
+      <c r="I2" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="13" t="s">
+      <c r="J2" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="13" t="s">
+      <c r="K2" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="13" t="s">
+      <c r="L2" s="14" t="s">
         <v>129</v>
       </c>
-      <c r="M2" s="13" t="s">
+      <c r="M2" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="N2" s="13" t="s">
+      <c r="N2" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="O2" s="13" t="s">
+      <c r="O2" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="P2" s="13"/>
-      <c r="Q2" s="13" t="s">
+      <c r="P2" s="14"/>
+      <c r="Q2" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="R2" s="13"/>
-      <c r="S2" s="13" t="s">
+      <c r="R2" s="14"/>
+      <c r="S2" s="14" t="s">
         <v>193</v>
       </c>
-      <c r="T2" s="13" t="s">
+      <c r="T2" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="U2" s="13" t="s">
+      <c r="U2" s="14" t="s">
         <v>195</v>
       </c>
-      <c r="V2" s="13" t="s">
+      <c r="V2" s="14" t="s">
         <v>196</v>
       </c>
-      <c r="W2" s="13" t="s">
+      <c r="W2" s="14" t="s">
         <v>197</v>
       </c>
-      <c r="X2" s="13" t="s">
+      <c r="X2" s="14" t="s">
         <v>198</v>
       </c>
-      <c r="Y2" s="13" t="s">
+      <c r="Y2" s="14" t="s">
         <v>199</v>
       </c>
-      <c r="Z2" s="13" t="s">
+      <c r="Z2" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="AA2" s="13" t="s">
+      <c r="AA2" s="14" t="s">
         <v>201</v>
       </c>
     </row>
     <row r="3" spans="1:27" ht="25">
-      <c r="A3" s="13"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
-      <c r="L3" s="13"/>
-      <c r="M3" s="13"/>
-      <c r="N3" s="13"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
+      <c r="L3" s="14"/>
+      <c r="M3" s="14"/>
+      <c r="N3" s="14"/>
       <c r="O3" s="1" t="s">
         <v>16</v>
       </c>
@@ -7146,15 +7143,15 @@
       <c r="R3" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="S3" s="13"/>
-      <c r="T3" s="13"/>
-      <c r="U3" s="13"/>
-      <c r="V3" s="13"/>
-      <c r="W3" s="13"/>
-      <c r="X3" s="13"/>
-      <c r="Y3" s="13"/>
-      <c r="Z3" s="13"/>
-      <c r="AA3" s="13"/>
+      <c r="S3" s="14"/>
+      <c r="T3" s="14"/>
+      <c r="U3" s="14"/>
+      <c r="V3" s="14"/>
+      <c r="W3" s="14"/>
+      <c r="X3" s="14"/>
+      <c r="Y3" s="14"/>
+      <c r="Z3" s="14"/>
+      <c r="AA3" s="14"/>
     </row>
     <row r="4" spans="1:27">
       <c r="A4" s="2" t="s">
@@ -8065,12 +8062,16 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="AA2:AA3"/>
-    <mergeCell ref="V2:V3"/>
-    <mergeCell ref="W2:W3"/>
-    <mergeCell ref="X2:X3"/>
-    <mergeCell ref="Y2:Y3"/>
-    <mergeCell ref="Z2:Z3"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:J3"/>
     <mergeCell ref="K2:K3"/>
     <mergeCell ref="O2:P2"/>
     <mergeCell ref="S2:S3"/>
@@ -8080,16 +8081,12 @@
     <mergeCell ref="L2:L3"/>
     <mergeCell ref="M2:M3"/>
     <mergeCell ref="N2:N3"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:J3"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="AA2:AA3"/>
+    <mergeCell ref="V2:V3"/>
+    <mergeCell ref="W2:W3"/>
+    <mergeCell ref="X2:X3"/>
+    <mergeCell ref="Y2:Y3"/>
+    <mergeCell ref="Z2:Z3"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.2" top="0.12013890000000001" bottom="0" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape"/>
@@ -8138,89 +8135,89 @@
       <c r="I1" s="9"/>
       <c r="J1" s="9"/>
       <c r="K1" s="9"/>
-      <c r="L1" s="13" t="s">
+      <c r="L1" s="14" t="s">
         <v>244</v>
       </c>
-      <c r="M1" s="13"/>
-      <c r="N1" s="13"/>
-      <c r="O1" s="13"/>
-      <c r="P1" s="13"/>
-      <c r="Q1" s="13"/>
-      <c r="R1" s="13"/>
-      <c r="S1" s="13"/>
+      <c r="M1" s="14"/>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="14"/>
+      <c r="Q1" s="14"/>
+      <c r="R1" s="14"/>
+      <c r="S1" s="14"/>
     </row>
     <row r="2" spans="1:19">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="D2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="G2" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="I2" s="13" t="s">
+      <c r="I2" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="J2" s="13" t="s">
+      <c r="J2" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="K2" s="13" t="s">
+      <c r="K2" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="13" t="s">
+      <c r="L2" s="14" t="s">
         <v>245</v>
       </c>
-      <c r="M2" s="13" t="s">
+      <c r="M2" s="14" t="s">
         <v>246</v>
       </c>
-      <c r="N2" s="13" t="s">
+      <c r="N2" s="14" t="s">
         <v>247</v>
       </c>
-      <c r="O2" s="13" t="s">
+      <c r="O2" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="P2" s="13" t="s">
+      <c r="P2" s="14" t="s">
         <v>248</v>
       </c>
-      <c r="Q2" s="13" t="s">
+      <c r="Q2" s="14" t="s">
         <v>249</v>
       </c>
-      <c r="R2" s="13"/>
-      <c r="S2" s="13"/>
+      <c r="R2" s="14"/>
+      <c r="S2" s="14"/>
     </row>
     <row r="3" spans="1:19" ht="25">
-      <c r="A3" s="13"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="D3" s="13"/>
-      <c r="E3" s="13"/>
-      <c r="F3" s="13"/>
-      <c r="G3" s="13"/>
-      <c r="H3" s="13"/>
-      <c r="I3" s="13"/>
-      <c r="J3" s="13"/>
-      <c r="K3" s="13"/>
-      <c r="L3" s="13"/>
-      <c r="M3" s="13"/>
-      <c r="N3" s="13"/>
-      <c r="O3" s="13"/>
-      <c r="P3" s="13"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
+      <c r="K3" s="14"/>
+      <c r="L3" s="14"/>
+      <c r="M3" s="14"/>
+      <c r="N3" s="14"/>
+      <c r="O3" s="14"/>
+      <c r="P3" s="14"/>
       <c r="Q3" s="1" t="s">
         <v>250</v>
       </c>
@@ -8364,7 +8361,7 @@
         <v>44635.468206018515</v>
       </c>
       <c r="L6" s="12" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="M6" s="7" t="s">
         <v>260</v>
@@ -8415,7 +8412,7 @@
         <v>44635.468206018515</v>
       </c>
       <c r="L7" s="12" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="M7" s="7" t="s">
         <v>260</v>
@@ -9176,7 +9173,7 @@
         <v>44587.558275462958</v>
       </c>
       <c r="L22" s="12" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="M22" s="7" t="s">
         <v>180</v>
@@ -9282,7 +9279,7 @@
         <v>44621.497152777774</v>
       </c>
       <c r="L24" s="12" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="M24" s="7" t="s">
         <v>304</v>
@@ -9335,7 +9332,7 @@
         <v>44621.497152777774</v>
       </c>
       <c r="L25" s="12" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="M25" s="7" t="s">
         <v>308</v>
@@ -9388,7 +9385,7 @@
         <v>44621.497152777774</v>
       </c>
       <c r="L26" s="12" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="M26" s="7" t="s">
         <v>300</v>
@@ -9490,7 +9487,7 @@
         <v>44631.713113425925</v>
       </c>
       <c r="L28" s="12" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="M28" s="7" t="s">
         <v>313</v>
@@ -9541,7 +9538,7 @@
         <v>44631.713113425925</v>
       </c>
       <c r="L29" s="12" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
       <c r="M29" s="7" t="s">
         <v>316</v>
@@ -9563,6 +9560,16 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="F2:F3"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I2:I3"/>
+    <mergeCell ref="J2:J3"/>
     <mergeCell ref="K2:K3"/>
     <mergeCell ref="L1:S1"/>
     <mergeCell ref="L2:L3"/>
@@ -9571,16 +9578,6 @@
     <mergeCell ref="O2:O3"/>
     <mergeCell ref="P2:P3"/>
     <mergeCell ref="Q2:S2"/>
-    <mergeCell ref="F2:F3"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I2:I3"/>
-    <mergeCell ref="J2:J3"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
-    <mergeCell ref="E2:E3"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.2" top="0.12013890000000001" bottom="0" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape"/>
@@ -9961,98 +9958,98 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="14" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="13" t="s">
+      <c r="D1" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="13" t="s">
+      <c r="E1" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="G1" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="I1" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="13" t="s">
+      <c r="J1" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="13" t="s">
+      <c r="K1" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="13" t="s">
+      <c r="L1" s="14" t="s">
         <v>245</v>
       </c>
-      <c r="M1" s="13" t="s">
+      <c r="M1" s="14" t="s">
         <v>337</v>
       </c>
-      <c r="N1" s="13" t="s">
+      <c r="N1" s="14" t="s">
         <v>338</v>
       </c>
-      <c r="O1" s="13" t="s">
+      <c r="O1" s="14" t="s">
         <v>339</v>
       </c>
-      <c r="P1" s="13" t="s">
+      <c r="P1" s="14" t="s">
         <v>321</v>
       </c>
-      <c r="Q1" s="13" t="s">
+      <c r="Q1" s="14" t="s">
         <v>340</v>
       </c>
-      <c r="R1" s="13"/>
-      <c r="S1" s="13" t="s">
+      <c r="R1" s="14"/>
+      <c r="S1" s="14" t="s">
         <v>341</v>
       </c>
-      <c r="T1" s="13" t="s">
+      <c r="T1" s="14" t="s">
         <v>342</v>
       </c>
-      <c r="U1" s="13" t="s">
+      <c r="U1" s="14" t="s">
         <v>343</v>
       </c>
-      <c r="V1" s="13" t="s">
+      <c r="V1" s="14" t="s">
         <v>344</v>
       </c>
     </row>
     <row r="2" spans="1:22">
-      <c r="A2" s="13"/>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="G2" s="13"/>
-      <c r="H2" s="13"/>
-      <c r="I2" s="13"/>
-      <c r="J2" s="13"/>
-      <c r="K2" s="13"/>
-      <c r="L2" s="13"/>
-      <c r="M2" s="13"/>
-      <c r="N2" s="13"/>
-      <c r="O2" s="13"/>
-      <c r="P2" s="13"/>
+      <c r="A2" s="14"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
+      <c r="D2" s="14"/>
+      <c r="E2" s="14"/>
+      <c r="F2" s="14"/>
+      <c r="G2" s="14"/>
+      <c r="H2" s="14"/>
+      <c r="I2" s="14"/>
+      <c r="J2" s="14"/>
+      <c r="K2" s="14"/>
+      <c r="L2" s="14"/>
+      <c r="M2" s="14"/>
+      <c r="N2" s="14"/>
+      <c r="O2" s="14"/>
+      <c r="P2" s="14"/>
       <c r="Q2" s="1" t="s">
         <v>345</v>
       </c>
       <c r="R2" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="S2" s="13"/>
-      <c r="T2" s="13"/>
-      <c r="U2" s="13"/>
-      <c r="V2" s="13"/>
+      <c r="S2" s="14"/>
+      <c r="T2" s="14"/>
+      <c r="U2" s="14"/>
+      <c r="V2" s="14"/>
     </row>
     <row r="3" spans="1:22">
       <c r="A3" s="2" t="s">
@@ -10168,6 +10165,16 @@
     </row>
   </sheetData>
   <mergeCells count="21">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:G2"/>
+    <mergeCell ref="H1:H2"/>
+    <mergeCell ref="I1:I2"/>
+    <mergeCell ref="J1:J2"/>
     <mergeCell ref="K1:K2"/>
     <mergeCell ref="V1:V2"/>
     <mergeCell ref="U1:U2"/>
@@ -10179,16 +10186,6 @@
     <mergeCell ref="P1:P2"/>
     <mergeCell ref="S1:S2"/>
     <mergeCell ref="T1:T2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:G2"/>
-    <mergeCell ref="H1:H2"/>
-    <mergeCell ref="I1:I2"/>
-    <mergeCell ref="J1:J2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="E1:E2"/>
   </mergeCells>
   <pageMargins left="0.3" right="0.2" top="0.12013890000000001" bottom="0" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape"/>

</xml_diff>